<commit_message>
planilha: tira "confiável" do selo; o selo diz de onde veio o número
A nota do topo e a instrução 4 diziam "(confiável)" e "Confiável pra aprovar
direto" em toda planilha, o contrário do /dados e da revisão de arquiteto ou
engenheiro habilitado. Exemplo público regerado.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/exemplos/quantitativo-exemplo-aiarq.xlsx
+++ b/exemplos/quantitativo-exemplo-aiarq.xlsx
@@ -945,7 +945,7 @@
     <row r="3">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>Cada item traz na coluna OBSERVAÇÕES um selo de status: "✓ MEDIDO do CAD" (confiável) ou "⚠ ESTIMADO — revisar". A cor é só reforço — fundo BRANCO = medido · LARANJA = estimado · CINZA = metadado · ROXO = custo indireto/gestão. Coluna AMARELA = preencher preço. Itens ⚠ ESTIMADO e os roxos exigem revisão antes de fechar o orçamento.</t>
+          <t>Cada item traz na coluna OBSERVAÇÕES um selo de status: "✓ MEDIDO do CAD" (saiu do desenho) ou "⚠ ESTIMADO — revisar". A cor é só reforço — fundo BRANCO = medido · LARANJA = estimado · CINZA = metadado · ROXO = custo indireto/gestão. Coluna AMARELA = preencher preço. Itens ⚠ ESTIMADO e os roxos exigem revisão antes de fechar o orçamento.</t>
         </is>
       </c>
     </row>
@@ -3947,7 +3947,7 @@
     <row r="128">
       <c r="A128" s="62" t="inlineStr">
         <is>
-          <t>4. Itens em BRANCO: quantidade medida/contada diretamente do arquivo (bloco, hachura, linha). Confiável pra aprovar direto.</t>
+          <t>4. Itens em BRANCO: quantidade medida/contada diretamente do arquivo (bloco, hachura, linha). O selo diz de onde veio o número; a conferência final é sua.</t>
         </is>
       </c>
     </row>

</xml_diff>